<commit_message>
J apublica les relations
</commit_message>
<xml_diff>
--- a/temporal/cameresBertaPerEntities.xlsx
+++ b/temporal/cameresBertaPerEntities.xlsx
@@ -12,15 +12,15 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="11580" windowHeight="7065" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja4" sheetId="4" r:id="rId2"/>
+    <sheet name="Dades diferents" sheetId="1" r:id="rId1"/>
+    <sheet name="Dades compartides" sheetId="5" r:id="rId2"/>
     <sheet name="1" sheetId="3" r:id="rId3"/>
-    <sheet name="Sensor" sheetId="2" r:id="rId4"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sensor" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="exempleCameresBerta_1" localSheetId="1">Hoja4!$A$1:$CK$21</definedName>
+    <definedName name="exempleCameresBerta_1" localSheetId="3">Hoja4!$A$1:$CK$21</definedName>
     <definedName name="ObservationsEspecies" localSheetId="2">'1'!$A$1:$J$8</definedName>
-    <definedName name="ObservationsFotos" localSheetId="3">Sensor!$A$1:$H$21</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,140 +31,8 @@
 </workbook>
 </file>
 
-<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" name="exempleCameresBerta" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="850" sourceFile="C:\inetpub\wwwroot\TAPIS\temporal\csv\exempleCameresBerta.csv" thousands=" " tab="0" semicolon="1">
-      <textFields count="89">
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-      </textFields>
-    </textPr>
-  </connection>
-  <connection id="2" name="ObservationsEspecies" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="850" sourceFile="C:\Users\m.olive\Downloads\ObservationsEspecies.csv" thousands=" " tab="0" semicolon="1">
-      <textFields count="10">
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-      </textFields>
-    </textPr>
-  </connection>
-  <connection id="3" name="ObservationsFotos" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="850" sourceFile="C:\Users\m.olive\Downloads\ObservationsFotos.csv" thousands=" " tab="0" semicolon="1">
-      <textFields count="10">
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-      </textFields>
-    </textPr>
-  </connection>
-</connections>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="410">
   <si>
     <t>@iot.selfLink</t>
   </si>
@@ -1208,13 +1076,199 @@
   </si>
   <si>
     <t>OBS020_Identification</t>
+  </si>
+  <si>
+    <t>Foto_Sensor.name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">encodingType: </t>
+  </si>
+  <si>
+    <t>Foto</t>
+  </si>
+  <si>
+    <t>application/json</t>
+  </si>
+  <si>
+    <t>metadata</t>
+  </si>
+  <si>
+    <t>CameraTrap_01</t>
+  </si>
+  <si>
+    <t>CameraTrap_02</t>
+  </si>
+  <si>
+    <t>CameraTrap_03</t>
+  </si>
+  <si>
+    <t>Motion-activated wildlife camera used to capture images of animals in their natural habitat.</t>
+  </si>
+  <si>
+    <t>{ "manufacturer": "Browning Trail Cameras", "model": "Strike Force Pro DCL", "sensorType": "Motion-activated wildlife camera", "imageResolution": "26 MP", "videoResolution": "1920 x 1080 (Full HD)", "dayNightCapture": true, "infraredIllumination": true, "motionDetectionRange": "100 ft", "triggerSpeed": "0.15 seconds", "application": "Wildlife monitoring and biodiversity observation" }</t>
+  </si>
+  <si>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description: </t>
+  </si>
+  <si>
+    <t>Person</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>WildlifeIdentifier_01</t>
+  </si>
+  <si>
+    <t>Person responsible for identifying and validating wildlife species from camera trap images, including the review and verification of species observations.</t>
+  </si>
+  <si>
+    <t>{ "identifier": "WildlifeIdentifier_01", "type": "Human observer", "role": "Wildlife species identifier", "responsibilities": [ "Species identification", "Image review", "Identification validation" ], "identificationMethod": "Visual identification from camera trap images" }</t>
+  </si>
+  <si>
+    <t>ObservedProperty</t>
+  </si>
+  <si>
+    <t>definition</t>
+  </si>
+  <si>
+    <t>properties</t>
+  </si>
+  <si>
+    <t>WildlifeImage</t>
+  </si>
+  <si>
+    <t>Wildlife image captured by a camera trap and stored at a URL</t>
+  </si>
+  <si>
+    <t>Digital photograph captured by a camera trap to document wildlife presence and behaviour. The image is stored externally and referenced through a URL</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>SpeciesIdentification</t>
+  </si>
+  <si>
+    <t>Taxonomic identification of a wildlife species observed in a camera trap image.</t>
+  </si>
+  <si>
+    <t>Species identified from a camera trap image by a human observer. The result records the assigned taxon and may include the confidence level and validation status.</t>
+  </si>
+  <si>
+    <t>Thing</t>
+  </si>
+  <si>
+    <t>Foto_Thing.name</t>
+  </si>
+  <si>
+    <t>Motion-activated camera trap used for wildlife monitoring.</t>
+  </si>
+  <si>
+    <t>{"deviceType":"Camera trap","manufacturer":"Browning Trail Cameras","model":"Strike Force Pro DCL","modelNumber":"BTC-5DCL","imageResolutionMP":26,"videoResolution":"1920x1080","triggerSpeedSeconds":0.15,"motionDetectionRangeMeters":30.48,"infraredNightVision":true,"fieldOfViewDegrees":54,"storageType":"SDXC","maxStorageCapacityGB":512,"powerSource":"6 AA batteries","purpose":"Wildlife monitoring","status":"Active"}</t>
+  </si>
+  <si>
+    <t>Human observer responsible for identifying and validating wildlife species from camera trap images.</t>
+  </si>
+  <si>
+    <t>{"entityType":"Human observer","role":"Wildlife species identifier","identificationMethods":["Visual identification","Camera trap image analysis"],"responsibilities":["Species identification","Image review","Taxonomic validation"],"expertise":"Wildlife ecology and species identification","organization":"Wildlife Monitoring Project","status":"Active"}</t>
+  </si>
+  <si>
+    <t>Datastream</t>
+  </si>
+  <si>
+    <t>unitOfMEasurement</t>
+  </si>
+  <si>
+    <t>Camera trap photograph</t>
+  </si>
+  <si>
+    <t>Photographs captured automatically by motion-activated camera traps for wildlife monitoring, species detection and documentation of animal behaviour in natural habitats.</t>
+  </si>
+  <si>
+    <t>{"name":"image","symbol":"img","definition":"Digital image"}</t>
+  </si>
+  <si>
+    <t>{"captureMethod":"camera_trap","automation":"motion-activated","mediaType":"image/jpeg","storageType":"URL","purpose":"Wildlife monitoring"}</t>
+  </si>
+  <si>
+    <t>Taxon identification</t>
+  </si>
+  <si>
+    <t>Taxonomic identification of wildlife species based on the visual analysis of camera trap images or field photographs by a human observer</t>
+  </si>
+  <si>
+    <t>{}</t>
+  </si>
+  <si>
+    <t>{"identificationMethod":"Human visual identification","purpose":"Wildlife monitoring","validationStatus":"Validated","inputDataType":"Photograph"}</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Location.name</t>
+  </si>
+  <si>
+    <t>Location.description</t>
+  </si>
+  <si>
+    <t>Location.location</t>
+  </si>
+  <si>
+    <t>Sant Jeroni</t>
+  </si>
+  <si>
+    <t>application/geo+json</t>
+  </si>
+  <si>
+    <t>{"type":"Point","coordinates":[1.81129,41.60534]}</t>
+  </si>
+  <si>
+    <t>Observation point near Sant Jeroni</t>
+  </si>
+  <si>
+    <t>locaion.properties</t>
+  </si>
+  <si>
+    <t>{"mountain":"Montserrat","habitat":"Rocky mountain","altitudeMeters":1236,"locationType":"Wildlife monitoring site"}</t>
+  </si>
+  <si>
+    <t>Ermita de Sant Joan</t>
+  </si>
+  <si>
+    <t>Observation point near Ermita de Sant Joan</t>
+  </si>
+  <si>
+    <t>{"type":"Point","coordinates":[1.8097,41.5927]}</t>
+  </si>
+  <si>
+    <t>{"mountain":"Montserrat","habitat":"Mediterranean rocky mountain","locationType":"Wildlife monitoring site","nearbyLandmark":"Ermita de Sant Joan"}</t>
+  </si>
+  <si>
+    <t>Ermita de Santa Magdalena</t>
+  </si>
+  <si>
+    <t>Observation point near Ermita de Santa Magdalena</t>
+  </si>
+  <si>
+    <t>{"type":"Point","coordinates":[1.8130,41.5920]}</t>
+  </si>
+  <si>
+    <t>{"mountain":"Montserrat","habitat":"Rocky Mediterranean mountain","locationType":"Wildlife monitoring site","nearbyLandmark":"Ermita de Santa Magdalena"}</t>
+  </si>
+  <si>
+    <t>locATION</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1230,13 +1284,48 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10.199999999999999"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1252,9 +1341,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1271,18 +1375,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="exempleCameresBerta_1" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
-<file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ObservationsEspecies" connectionId="2" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
-<file path=xl/queryTables/queryTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ObservationsFotos" connectionId="3" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1548,23 +1640,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C44"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I1048576"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="98.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="76.42578125" customWidth="1"/>
     <col min="3" max="3" width="35.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="27.140625" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.140625" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" customWidth="1"/>
     <col min="8" max="8" width="31.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1574,8 +1666,26 @@
       <c r="C1" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E1" t="s">
+        <v>376</v>
+      </c>
+      <c r="F1" t="s">
+        <v>392</v>
+      </c>
+      <c r="G1" t="s">
+        <v>393</v>
+      </c>
+      <c r="H1" t="s">
+        <v>394</v>
+      </c>
+      <c r="I1" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1585,8 +1695,26 @@
       <c r="C2" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H2" t="s">
+        <v>397</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1596,8 +1724,26 @@
       <c r="C3" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H3" t="s">
+        <v>397</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1607,8 +1753,26 @@
       <c r="C4" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H4" t="s">
+        <v>397</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1618,8 +1782,26 @@
       <c r="C5" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H5" t="s">
+        <v>397</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -1629,8 +1811,26 @@
       <c r="C6" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="H6" t="s">
+        <v>403</v>
+      </c>
+      <c r="I6" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -1640,8 +1840,26 @@
       <c r="C7" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="G7" t="s">
+        <v>402</v>
+      </c>
+      <c r="H7" t="s">
+        <v>403</v>
+      </c>
+      <c r="I7" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -1651,8 +1869,26 @@
       <c r="C8" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="G8" t="s">
+        <v>402</v>
+      </c>
+      <c r="H8" t="s">
+        <v>403</v>
+      </c>
+      <c r="I8" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -1662,8 +1898,26 @@
       <c r="C9" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="G9" t="s">
+        <v>402</v>
+      </c>
+      <c r="H9" t="s">
+        <v>403</v>
+      </c>
+      <c r="I9" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -1673,8 +1927,26 @@
       <c r="C10" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G10" t="s">
+        <v>406</v>
+      </c>
+      <c r="H10" t="s">
+        <v>407</v>
+      </c>
+      <c r="I10" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>68</v>
       </c>
@@ -1684,8 +1956,26 @@
       <c r="C11" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G11" t="s">
+        <v>406</v>
+      </c>
+      <c r="H11" t="s">
+        <v>407</v>
+      </c>
+      <c r="I11" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>68</v>
       </c>
@@ -1695,8 +1985,26 @@
       <c r="C12" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G12" t="s">
+        <v>406</v>
+      </c>
+      <c r="H12" t="s">
+        <v>407</v>
+      </c>
+      <c r="I12" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>81</v>
       </c>
@@ -1706,8 +2014,26 @@
       <c r="C13" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G13" t="s">
+        <v>406</v>
+      </c>
+      <c r="H13" t="s">
+        <v>407</v>
+      </c>
+      <c r="I13" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>81</v>
       </c>
@@ -1717,8 +2043,26 @@
       <c r="C14" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G14" t="s">
+        <v>406</v>
+      </c>
+      <c r="H14" t="s">
+        <v>407</v>
+      </c>
+      <c r="I14" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -1728,8 +2072,26 @@
       <c r="C15" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G15" t="s">
+        <v>406</v>
+      </c>
+      <c r="H15" t="s">
+        <v>407</v>
+      </c>
+      <c r="I15" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>81</v>
       </c>
@@ -1739,8 +2101,26 @@
       <c r="C16" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G16" t="s">
+        <v>406</v>
+      </c>
+      <c r="H16" t="s">
+        <v>407</v>
+      </c>
+      <c r="I16" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>106</v>
       </c>
@@ -1750,8 +2130,26 @@
       <c r="C17" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G17" t="s">
+        <v>406</v>
+      </c>
+      <c r="H17" t="s">
+        <v>407</v>
+      </c>
+      <c r="I17" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>106</v>
       </c>
@@ -1761,8 +2159,26 @@
       <c r="C18" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G18" t="s">
+        <v>406</v>
+      </c>
+      <c r="H18" t="s">
+        <v>407</v>
+      </c>
+      <c r="I18" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -1772,8 +2188,26 @@
       <c r="C19" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G19" t="s">
+        <v>406</v>
+      </c>
+      <c r="H19" t="s">
+        <v>407</v>
+      </c>
+      <c r="I19" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>125</v>
       </c>
@@ -1783,8 +2217,26 @@
       <c r="C20" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G20" t="s">
+        <v>406</v>
+      </c>
+      <c r="H20" t="s">
+        <v>407</v>
+      </c>
+      <c r="I20" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>125</v>
       </c>
@@ -1794,190 +2246,752 @@
       <c r="C21" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>2</v>
-      </c>
-      <c r="B24" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>10</v>
-      </c>
-      <c r="B28" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>36</v>
-      </c>
-      <c r="B29" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>61</v>
-      </c>
-      <c r="B33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>68</v>
-      </c>
-      <c r="B35" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>81</v>
-      </c>
-      <c r="B36" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>81</v>
-      </c>
-      <c r="B37" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>81</v>
-      </c>
-      <c r="B38" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>81</v>
-      </c>
-      <c r="B39" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>106</v>
-      </c>
-      <c r="B40" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>106</v>
-      </c>
-      <c r="B41" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>106</v>
-      </c>
-      <c r="B42" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>125</v>
-      </c>
-      <c r="B43" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>125</v>
-      </c>
-      <c r="B44" t="s">
-        <v>139</v>
+      <c r="D21" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="G21" t="s">
+        <v>406</v>
+      </c>
+      <c r="H21" t="s">
+        <v>407</v>
+      </c>
+      <c r="I21" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="B26" s="1"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="B30" s="1"/>
+    </row>
+    <row r="1048576" spans="8:8">
+      <c r="H1048576" t="s">
+        <v>403</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B26" r:id="rId1"/>
-    <hyperlink ref="C3" r:id="rId2"/>
-    <hyperlink ref="B30" r:id="rId3"/>
+    <hyperlink ref="C3" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="107.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>360</v>
+      </c>
+      <c r="B4" t="s">
+        <v>358</v>
+      </c>
+      <c r="C4" t="s">
+        <v>361</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>360</v>
+      </c>
+      <c r="B5" t="s">
+        <v>358</v>
+      </c>
+      <c r="C5" t="s">
+        <v>359</v>
+      </c>
+      <c r="D5" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>360</v>
+      </c>
+      <c r="B6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C6" t="s">
+        <v>349</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B7" t="s">
+        <v>358</v>
+      </c>
+      <c r="C7" t="s">
+        <v>352</v>
+      </c>
+      <c r="D7" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="17.25">
+      <c r="A9" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="17.25">
+      <c r="A10" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="17.25">
+      <c r="A11" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>360</v>
+      </c>
+      <c r="B12" t="s">
+        <v>365</v>
+      </c>
+      <c r="C12" t="s">
+        <v>361</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="17.25">
+      <c r="A13" t="s">
+        <v>360</v>
+      </c>
+      <c r="B13" t="s">
+        <v>365</v>
+      </c>
+      <c r="C13" t="s">
+        <v>366</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="17.25">
+      <c r="A14" t="s">
+        <v>360</v>
+      </c>
+      <c r="B14" t="s">
+        <v>365</v>
+      </c>
+      <c r="C14" t="s">
+        <v>359</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="17.25">
+      <c r="A15" t="s">
+        <v>360</v>
+      </c>
+      <c r="B15" t="s">
+        <v>365</v>
+      </c>
+      <c r="C15" t="s">
+        <v>367</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="17.25">
+      <c r="A17" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>360</v>
+      </c>
+      <c r="B18" t="s">
+        <v>375</v>
+      </c>
+      <c r="C18" t="s">
+        <v>361</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>360</v>
+      </c>
+      <c r="B19" t="s">
+        <v>375</v>
+      </c>
+      <c r="C19" t="s">
+        <v>359</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="17.25">
+      <c r="A20" t="s">
+        <v>360</v>
+      </c>
+      <c r="B20" t="s">
+        <v>375</v>
+      </c>
+      <c r="C20" t="s">
+        <v>367</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="17.25">
+      <c r="A24" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>360</v>
+      </c>
+      <c r="B25" t="s">
+        <v>381</v>
+      </c>
+      <c r="C25" t="s">
+        <v>361</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>360</v>
+      </c>
+      <c r="B26" t="s">
+        <v>381</v>
+      </c>
+      <c r="C26" t="s">
+        <v>359</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>360</v>
+      </c>
+      <c r="B27" t="s">
+        <v>381</v>
+      </c>
+      <c r="C27" t="s">
+        <v>382</v>
+      </c>
+      <c r="D27" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="17.25">
+      <c r="A28" t="s">
+        <v>360</v>
+      </c>
+      <c r="B28" t="s">
+        <v>381</v>
+      </c>
+      <c r="C28" t="s">
+        <v>367</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>409</v>
+      </c>
+      <c r="B29" t="s">
+        <v>391</v>
+      </c>
+      <c r="C29" t="s">
+        <v>349</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>396</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="73.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="79.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="69.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="80.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="70.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2">
+        <v>1393286</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H2" t="s">
+        <v>142</v>
+      </c>
+      <c r="I2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3">
+        <v>1393295</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>146</v>
+      </c>
+      <c r="G3" t="s">
+        <v>147</v>
+      </c>
+      <c r="H3" t="s">
+        <v>148</v>
+      </c>
+      <c r="I3" t="s">
+        <v>149</v>
+      </c>
+      <c r="J3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B4">
+        <v>1393296</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>152</v>
+      </c>
+      <c r="G4" t="s">
+        <v>153</v>
+      </c>
+      <c r="H4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I4" t="s">
+        <v>155</v>
+      </c>
+      <c r="J4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5">
+        <v>1393298</v>
+      </c>
+      <c r="C5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" t="s">
+        <v>159</v>
+      </c>
+      <c r="H5" t="s">
+        <v>160</v>
+      </c>
+      <c r="I5" t="s">
+        <v>161</v>
+      </c>
+      <c r="J5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6">
+        <v>1393303</v>
+      </c>
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>164</v>
+      </c>
+      <c r="G6" t="s">
+        <v>165</v>
+      </c>
+      <c r="H6" t="s">
+        <v>166</v>
+      </c>
+      <c r="I6" t="s">
+        <v>167</v>
+      </c>
+      <c r="J6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7">
+        <v>1393308</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>170</v>
+      </c>
+      <c r="G7" t="s">
+        <v>171</v>
+      </c>
+      <c r="H7" t="s">
+        <v>172</v>
+      </c>
+      <c r="I7" t="s">
+        <v>173</v>
+      </c>
+      <c r="J7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8">
+        <v>1393312</v>
+      </c>
+      <c r="C8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" t="s">
+        <v>139</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>176</v>
+      </c>
+      <c r="G8" t="s">
+        <v>177</v>
+      </c>
+      <c r="H8" t="s">
+        <v>178</v>
+      </c>
+      <c r="I8" t="s">
+        <v>179</v>
+      </c>
+      <c r="J8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CK21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
@@ -2329,7 +3343,7 @@
     <col min="399" max="399" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:89">
       <c r="A1" t="s">
         <v>218</v>
       </c>
@@ -2598,7 +3612,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="2" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:89">
       <c r="A2" t="s">
         <v>194</v>
       </c>
@@ -2651,7 +3665,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="3" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:89">
       <c r="A3" t="s">
         <v>195</v>
       </c>
@@ -2704,7 +3718,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:89">
       <c r="A4" t="s">
         <v>196</v>
       </c>
@@ -2757,7 +3771,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="5" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:89">
       <c r="A5" t="s">
         <v>197</v>
       </c>
@@ -2810,7 +3824,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="6" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:89">
       <c r="A6" t="s">
         <v>200</v>
       </c>
@@ -2863,7 +3877,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="7" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:89">
       <c r="A7" t="s">
         <v>201</v>
       </c>
@@ -2916,7 +3930,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="8" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:89">
       <c r="A8" t="s">
         <v>202</v>
       </c>
@@ -2969,7 +3983,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="9" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:89">
       <c r="A9" t="s">
         <v>203</v>
       </c>
@@ -3022,7 +4036,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="10" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:89">
       <c r="A10" t="s">
         <v>206</v>
       </c>
@@ -3075,7 +4089,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="11" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:89">
       <c r="A11" t="s">
         <v>207</v>
       </c>
@@ -3128,7 +4142,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="12" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:89">
       <c r="A12" t="s">
         <v>208</v>
       </c>
@@ -3181,7 +4195,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="13" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:89">
       <c r="A13" t="s">
         <v>209</v>
       </c>
@@ -3234,7 +4248,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="14" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:89">
       <c r="A14" t="s">
         <v>210</v>
       </c>
@@ -3287,7 +4301,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="15" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:89">
       <c r="A15" t="s">
         <v>211</v>
       </c>
@@ -3340,7 +4354,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="16" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:89">
       <c r="A16" t="s">
         <v>212</v>
       </c>
@@ -3393,7 +4407,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="17" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:73">
       <c r="A17" t="s">
         <v>213</v>
       </c>
@@ -3446,7 +4460,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="18" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:73">
       <c r="A18" t="s">
         <v>214</v>
       </c>
@@ -3499,7 +4513,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="19" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:73">
       <c r="A19" t="s">
         <v>215</v>
       </c>
@@ -3552,7 +4566,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="20" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:73">
       <c r="A20" t="s">
         <v>216</v>
       </c>
@@ -3605,7 +4619,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="21" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:73">
       <c r="A21" t="s">
         <v>217</v>
       </c>
@@ -3660,291 +4674,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.5703125" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="73.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="79.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="69.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="80.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="70.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B2">
-        <v>1393286</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>140</v>
-      </c>
-      <c r="G2" t="s">
-        <v>141</v>
-      </c>
-      <c r="H2" t="s">
-        <v>142</v>
-      </c>
-      <c r="I2" t="s">
-        <v>143</v>
-      </c>
-      <c r="J2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B3">
-        <v>1393295</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>146</v>
-      </c>
-      <c r="G3" t="s">
-        <v>147</v>
-      </c>
-      <c r="H3" t="s">
-        <v>148</v>
-      </c>
-      <c r="I3" t="s">
-        <v>149</v>
-      </c>
-      <c r="J3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B4">
-        <v>1393296</v>
-      </c>
-      <c r="C4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" t="s">
-        <v>139</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>152</v>
-      </c>
-      <c r="G4" t="s">
-        <v>153</v>
-      </c>
-      <c r="H4" t="s">
-        <v>154</v>
-      </c>
-      <c r="I4" t="s">
-        <v>155</v>
-      </c>
-      <c r="J4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>157</v>
-      </c>
-      <c r="B5">
-        <v>1393298</v>
-      </c>
-      <c r="C5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" t="s">
-        <v>139</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>158</v>
-      </c>
-      <c r="G5" t="s">
-        <v>159</v>
-      </c>
-      <c r="H5" t="s">
-        <v>160</v>
-      </c>
-      <c r="I5" t="s">
-        <v>161</v>
-      </c>
-      <c r="J5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>163</v>
-      </c>
-      <c r="B6">
-        <v>1393303</v>
-      </c>
-      <c r="C6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" t="s">
-        <v>139</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="s">
-        <v>164</v>
-      </c>
-      <c r="G6" t="s">
-        <v>165</v>
-      </c>
-      <c r="H6" t="s">
-        <v>166</v>
-      </c>
-      <c r="I6" t="s">
-        <v>167</v>
-      </c>
-      <c r="J6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>169</v>
-      </c>
-      <c r="B7">
-        <v>1393308</v>
-      </c>
-      <c r="C7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>170</v>
-      </c>
-      <c r="G7" t="s">
-        <v>171</v>
-      </c>
-      <c r="H7" t="s">
-        <v>172</v>
-      </c>
-      <c r="I7" t="s">
-        <v>173</v>
-      </c>
-      <c r="J7" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>175</v>
-      </c>
-      <c r="B8">
-        <v>1393312</v>
-      </c>
-      <c r="C8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D8" t="s">
-        <v>139</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="s">
-        <v>176</v>
-      </c>
-      <c r="G8" t="s">
-        <v>177</v>
-      </c>
-      <c r="H8" t="s">
-        <v>178</v>
-      </c>
-      <c r="I8" t="s">
-        <v>179</v>
-      </c>
-      <c r="J8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="81.140625" bestFit="1" customWidth="1"/>
@@ -3956,7 +4689,7 @@
     <col min="8" max="8" width="70.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -3982,7 +4715,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -4008,7 +4741,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -4034,7 +4767,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -4060,7 +4793,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -4086,7 +4819,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -4112,7 +4845,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -4138,7 +4871,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -4164,7 +4897,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -4190,7 +4923,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -4216,7 +4949,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>68</v>
       </c>
@@ -4242,7 +4975,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>68</v>
       </c>
@@ -4268,7 +5001,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>81</v>
       </c>
@@ -4294,7 +5027,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>81</v>
       </c>
@@ -4320,7 +5053,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -4346,7 +5079,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
         <v>81</v>
       </c>
@@ -4372,7 +5105,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
         <v>106</v>
       </c>
@@ -4398,7 +5131,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
         <v>106</v>
       </c>
@@ -4424,7 +5157,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -4450,7 +5183,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
         <v>125</v>
       </c>
@@ -4476,7 +5209,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
         <v>125</v>
       </c>

</xml_diff>